<commit_message>
reviewed the annotations and redone the results
</commit_message>
<xml_diff>
--- a/2d/results/best_unet_filter_projection_max/best_unet.xlsx
+++ b/2d/results/best_unet_filter_projection_max/best_unet.xlsx
@@ -535,55 +535,55 @@
         <v>140</v>
       </c>
       <c r="C2" t="n">
-        <v>22.30488177424518</v>
+        <v>27.96217730846893</v>
       </c>
       <c r="D2" t="n">
-        <v>13.4105268197998</v>
+        <v>10.91520238217487</v>
       </c>
       <c r="E2" t="n">
-        <v>36.05318827440322</v>
+        <v>32.98297428769983</v>
       </c>
       <c r="F2" t="n">
-        <v>12.43499999999999</v>
+        <v>14.62875000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>11.01500000000001</v>
+        <v>13.07374999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>77.30782625323259</v>
+        <v>83.55387483534201</v>
       </c>
       <c r="I2" t="n">
-        <v>73.56799575902555</v>
+        <v>74.24957912338628</v>
       </c>
       <c r="J2" t="n">
-        <v>66.48496070541067</v>
+        <v>71.14949051117652</v>
       </c>
       <c r="K2" t="n">
-        <v>65.36818798161688</v>
+        <v>69.11765331664552</v>
       </c>
       <c r="L2" t="n">
-        <v>38.61670622929925</v>
+        <v>43.89191269470949</v>
       </c>
       <c r="M2" t="n">
-        <v>32.9013677527242</v>
+        <v>37.36642878306676</v>
       </c>
       <c r="N2" t="n">
-        <v>73.20945977126179</v>
+        <v>76.53471434584439</v>
       </c>
       <c r="O2" t="n">
-        <v>63.46307981811157</v>
+        <v>67.35215289803288</v>
       </c>
       <c r="P2" t="n">
-        <v>20.09375526408756</v>
+        <v>22.08736236055058</v>
       </c>
       <c r="Q2" t="n">
-        <v>18.00325208257791</v>
+        <v>16.38238186880578</v>
       </c>
       <c r="R2" t="n">
-        <v>16.90351524038223</v>
+        <v>12.06203644370811</v>
       </c>
       <c r="S2" t="n">
-        <v>19.450019751513</v>
+        <v>18.00065087058495</v>
       </c>
     </row>
     <row r="3">
@@ -596,55 +596,55 @@
         <v>141</v>
       </c>
       <c r="C3" t="n">
-        <v>14.14203984271407</v>
+        <v>18.60611049745686</v>
       </c>
       <c r="D3" t="n">
-        <v>7.42552982498719</v>
+        <v>7.141540968918891</v>
       </c>
       <c r="E3" t="n">
-        <v>29.3671181690799</v>
+        <v>35.53118769581308</v>
       </c>
       <c r="F3" t="n">
-        <v>21.72999999999999</v>
+        <v>26.33249999999999</v>
       </c>
       <c r="G3" t="n">
-        <v>16.1125</v>
+        <v>19.68125</v>
       </c>
       <c r="H3" t="n">
-        <v>81.54140052758477</v>
+        <v>95.29559276272958</v>
       </c>
       <c r="I3" t="n">
-        <v>88.39259018718707</v>
+        <v>90.92991806880724</v>
       </c>
       <c r="J3" t="n">
-        <v>72.46550903705845</v>
+        <v>80.16389461596786</v>
       </c>
       <c r="K3" t="n">
-        <v>78.73531609131953</v>
+        <v>82.56209784156408</v>
       </c>
       <c r="L3" t="n">
-        <v>55.1724568965349</v>
+        <v>61.84658438426492</v>
       </c>
       <c r="M3" t="n">
-        <v>44.30857704779064</v>
+        <v>51.00245092149984</v>
       </c>
       <c r="N3" t="n">
-        <v>80.47126816448217</v>
+        <v>88.96979824637121</v>
       </c>
       <c r="O3" t="n">
-        <v>71.98480742490042</v>
+        <v>77.6937095265762</v>
       </c>
       <c r="P3" t="n">
-        <v>13.07028439621102</v>
+        <v>17.91642944338606</v>
       </c>
       <c r="Q3" t="n">
-        <v>13.44106496313544</v>
+        <v>15.59328281681619</v>
       </c>
       <c r="R3" t="n">
-        <v>14.0035010370336</v>
+        <v>13.20064452036078</v>
       </c>
       <c r="S3" t="n">
-        <v>12.85144306717778</v>
+        <v>15.19957494431834</v>
       </c>
     </row>
     <row r="4">
@@ -657,55 +657,55 @@
         <v>149</v>
       </c>
       <c r="C4" t="n">
-        <v>10.20974965976008</v>
+        <v>12.37028615723304</v>
       </c>
       <c r="D4" t="n">
-        <v>8.4468494436315</v>
+        <v>11.66611791141456</v>
       </c>
       <c r="E4" t="n">
-        <v>18.10344827586206</v>
+        <v>18.81877174833061</v>
       </c>
       <c r="F4" t="n">
-        <v>11.31</v>
+        <v>13.29125</v>
       </c>
       <c r="G4" t="n">
-        <v>9.378750000000002</v>
+        <v>10.89999999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>81.94662897276496</v>
+        <v>86.12345789620852</v>
       </c>
       <c r="I4" t="n">
-        <v>74.47314952383846</v>
+        <v>72.6808090213641</v>
       </c>
       <c r="J4" t="n">
-        <v>72.40338389882065</v>
+        <v>77.93587107359487</v>
       </c>
       <c r="K4" t="n">
-        <v>66.00189391222042</v>
+        <v>61.53251173160414</v>
       </c>
       <c r="L4" t="n">
-        <v>33.55964838909966</v>
+        <v>40.18084120572889</v>
       </c>
       <c r="M4" t="n">
-        <v>28.23118842698621</v>
+        <v>34.32928778754375</v>
       </c>
       <c r="N4" t="n">
-        <v>76.63223864666881</v>
+        <v>77.25161810603063</v>
       </c>
       <c r="O4" t="n">
-        <v>67.418932800809</v>
+        <v>67.71124352720159</v>
       </c>
       <c r="P4" t="n">
-        <v>14.67230195877975</v>
+        <v>12.74397936990539</v>
       </c>
       <c r="Q4" t="n">
-        <v>16.11742144580922</v>
+        <v>15.08611031820745</v>
       </c>
       <c r="R4" t="n">
-        <v>17.72475099793851</v>
+        <v>17.846656832127</v>
       </c>
       <c r="S4" t="n">
-        <v>17.09240296174209</v>
+        <v>15.76979805046937</v>
       </c>
     </row>
     <row r="5">
@@ -718,55 +718,55 @@
         <v>160</v>
       </c>
       <c r="C5" t="n">
-        <v>19.72121115484191</v>
+        <v>21.35831983066659</v>
       </c>
       <c r="D5" t="n">
-        <v>13.37068834110539</v>
+        <v>9.832006129761428</v>
       </c>
       <c r="E5" t="n">
-        <v>39.67122657776761</v>
+        <v>26.96701676801179</v>
       </c>
       <c r="F5" t="n">
-        <v>10.9725</v>
+        <v>14.45000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>8.137500000000006</v>
+        <v>12.40125000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>69.20260110718382</v>
+        <v>79.4638282490845</v>
       </c>
       <c r="I5" t="n">
-        <v>67.75876327088623</v>
+        <v>70.44501401802685</v>
       </c>
       <c r="J5" t="n">
-        <v>55.49099025968088</v>
+        <v>65.38539592294292</v>
       </c>
       <c r="K5" t="n">
-        <v>52.73755777432247</v>
+        <v>60.46693311223913</v>
       </c>
       <c r="L5" t="n">
-        <v>36.23534186398688</v>
+        <v>43.8919126947095</v>
       </c>
       <c r="M5" t="n">
-        <v>31.80015723231569</v>
+        <v>36.9120576505835</v>
       </c>
       <c r="N5" t="n">
-        <v>66.6131556075825</v>
+        <v>72.52068670386403</v>
       </c>
       <c r="O5" t="n">
-        <v>51.61637337124722</v>
+        <v>59.6028522807424</v>
       </c>
       <c r="P5" t="n">
-        <v>25.02312602194904</v>
+        <v>19.88454058896328</v>
       </c>
       <c r="Q5" t="n">
-        <v>24.20075348449812</v>
+        <v>20.52722918411169</v>
       </c>
       <c r="R5" t="n">
-        <v>23.36409810714269</v>
+        <v>21.25043922588592</v>
       </c>
       <c r="S5" t="n">
-        <v>25.61551068154738</v>
+        <v>20.9887280334298</v>
       </c>
     </row>
     <row r="6">
@@ -779,55 +779,55 @@
         <v>170</v>
       </c>
       <c r="C6" t="n">
-        <v>14.86195575878171</v>
+        <v>15.86668041581076</v>
       </c>
       <c r="D6" t="n">
-        <v>5.293260550725834</v>
+        <v>10.25837370790761</v>
       </c>
       <c r="E6" t="n">
-        <v>18.52228435858337</v>
+        <v>15.74316463059921</v>
       </c>
       <c r="F6" t="n">
-        <v>14.75250000000001</v>
+        <v>17.25000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>12.30125</v>
+        <v>15.13625</v>
       </c>
       <c r="H6" t="n">
-        <v>81.54140052758477</v>
+        <v>92.76987657639737</v>
       </c>
       <c r="I6" t="n">
-        <v>74.72951224248692</v>
+        <v>81.51380251221264</v>
       </c>
       <c r="J6" t="n">
-        <v>62.93250352560273</v>
+        <v>67.36839021380874</v>
       </c>
       <c r="K6" t="n">
-        <v>64.77074957108339</v>
+        <v>62.04232426336073</v>
       </c>
       <c r="L6" t="n">
-        <v>42.5</v>
+        <v>52.17518567288477</v>
       </c>
       <c r="M6" t="n">
-        <v>38.73306081372863</v>
+        <v>45.34313619501854</v>
       </c>
       <c r="N6" t="n">
-        <v>72.95246740172672</v>
+        <v>81.89055195808612</v>
       </c>
       <c r="O6" t="n">
-        <v>60.47830189415044</v>
+        <v>58.91148020547439</v>
       </c>
       <c r="P6" t="n">
-        <v>26.21363450139479</v>
+        <v>29.5352083982154</v>
       </c>
       <c r="Q6" t="n">
-        <v>20.50289185187905</v>
+        <v>26.89365686538416</v>
       </c>
       <c r="R6" t="n">
-        <v>14.27159260047867</v>
+        <v>23.88733889077819</v>
       </c>
       <c r="S6" t="n">
-        <v>19.63160111597088</v>
+        <v>28.06071177096603</v>
       </c>
     </row>
     <row r="7">
@@ -840,55 +840,55 @@
         <v>184</v>
       </c>
       <c r="C7" t="n">
-        <v>12.74010748814477</v>
+        <v>11.42512760753906</v>
       </c>
       <c r="D7" t="n">
-        <v>10.95708768739162</v>
+        <v>12.26558550933254</v>
       </c>
       <c r="E7" t="n">
-        <v>30.32128514056221</v>
+        <v>42.53453772582358</v>
       </c>
       <c r="F7" t="n">
-        <v>13.0725</v>
+        <v>14.955</v>
       </c>
       <c r="G7" t="n">
-        <v>9.460000000000001</v>
+        <v>12.425</v>
       </c>
       <c r="H7" t="n">
-        <v>79.7699818227383</v>
+        <v>86.48843853371386</v>
       </c>
       <c r="I7" t="n">
-        <v>74.60898069267533</v>
+        <v>73.77838436832295</v>
       </c>
       <c r="J7" t="n">
-        <v>66.54697588921678</v>
+        <v>72.95375247374189</v>
       </c>
       <c r="K7" t="n">
-        <v>64.7012364642284</v>
+        <v>67.23280449304491</v>
       </c>
       <c r="L7" t="n">
-        <v>36.09016486523718</v>
+        <v>41.72529209005013</v>
       </c>
       <c r="M7" t="n">
-        <v>28.60069929215018</v>
+        <v>35.04639781775011</v>
       </c>
       <c r="N7" t="n">
-        <v>74.20284698042252</v>
+        <v>76.28277983922716</v>
       </c>
       <c r="O7" t="n">
-        <v>64.56488983960244</v>
+        <v>69.51618516575834</v>
       </c>
       <c r="P7" t="n">
-        <v>21.46190960664089</v>
+        <v>18.39811060195704</v>
       </c>
       <c r="Q7" t="n">
-        <v>18.83914541128517</v>
+        <v>19.06380961006474</v>
       </c>
       <c r="R7" t="n">
-        <v>15.93236047877639</v>
+        <v>19.84986129525687</v>
       </c>
       <c r="S7" t="n">
-        <v>19.63481648974178</v>
+        <v>16.81647104249954</v>
       </c>
     </row>
     <row r="8">
@@ -901,55 +901,55 @@
         <v>190</v>
       </c>
       <c r="C8" t="n">
-        <v>11.66635401219507</v>
+        <v>14.84687884974327</v>
       </c>
       <c r="D8" t="n">
-        <v>6.356962766358665</v>
+        <v>6.714576234617923</v>
       </c>
       <c r="E8" t="n">
-        <v>32.2371886522688</v>
+        <v>22.79151943462898</v>
       </c>
       <c r="F8" t="n">
-        <v>16.61124999999999</v>
+        <v>19.81</v>
       </c>
       <c r="G8" t="n">
-        <v>11.37749999999999</v>
+        <v>15.46750000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>90.15680784056188</v>
+        <v>101.3718402713495</v>
       </c>
       <c r="I8" t="n">
-        <v>83.67944789492819</v>
+        <v>86.64006001844645</v>
       </c>
       <c r="J8" t="n">
-        <v>69.01630242196404</v>
+        <v>80.85944595407516</v>
       </c>
       <c r="K8" t="n">
-        <v>70.36511919978534</v>
+        <v>76.05918747922567</v>
       </c>
       <c r="L8" t="n">
-        <v>40.0780488547035</v>
+        <v>46.51881339845202</v>
       </c>
       <c r="M8" t="n">
-        <v>33.55964838909967</v>
+        <v>40.92065493122026</v>
       </c>
       <c r="N8" t="n">
-        <v>84.60570311746129</v>
+        <v>91.40192831663893</v>
       </c>
       <c r="O8" t="n">
-        <v>67.8122407829147</v>
+        <v>75.871602065595</v>
       </c>
       <c r="P8" t="n">
-        <v>24.19147807513857</v>
+        <v>20.63995165804235</v>
       </c>
       <c r="Q8" t="n">
-        <v>20.47728025795765</v>
+        <v>17.32859851638831</v>
       </c>
       <c r="R8" t="n">
-        <v>16.47557819957555</v>
+        <v>13.45420182637774</v>
       </c>
       <c r="S8" t="n">
-        <v>20.42086606664304</v>
+        <v>17.66723215289666</v>
       </c>
     </row>
     <row r="9">
@@ -962,55 +962,55 @@
         <v>198</v>
       </c>
       <c r="C9" t="n">
-        <v>25.4606618071623</v>
+        <v>26.44385637970483</v>
       </c>
       <c r="D9" t="n">
-        <v>15.19950401445536</v>
+        <v>13.45259901807294</v>
       </c>
       <c r="E9" t="n">
-        <v>22.80382775119626</v>
+        <v>17.02836826901714</v>
       </c>
       <c r="F9" t="n">
-        <v>14.49875</v>
+        <v>16.87625000000001</v>
       </c>
       <c r="G9" t="n">
-        <v>11.7375</v>
+        <v>14.495</v>
       </c>
       <c r="H9" t="n">
-        <v>83.62116956847711</v>
+        <v>93.29523031752481</v>
       </c>
       <c r="I9" t="n">
-        <v>75.85842075867386</v>
+        <v>80.18883962248114</v>
       </c>
       <c r="J9" t="n">
-        <v>71.23377008133151</v>
+        <v>76.03453162872775</v>
       </c>
       <c r="K9" t="n">
-        <v>66.6126864793787</v>
+        <v>68.52919086053765</v>
       </c>
       <c r="L9" t="n">
-        <v>39.60113634733226</v>
+        <v>46.01086828130936</v>
       </c>
       <c r="M9" t="n">
-        <v>35.67211796347394</v>
+        <v>39.13118960624632</v>
       </c>
       <c r="N9" t="n">
-        <v>77.49354811853694</v>
+        <v>84.32415134467705</v>
       </c>
       <c r="O9" t="n">
-        <v>66.75046816315223</v>
+        <v>69.73969457919931</v>
       </c>
       <c r="P9" t="n">
-        <v>17.91085236863058</v>
+        <v>19.38704205296404</v>
       </c>
       <c r="Q9" t="n">
-        <v>17.04654033627144</v>
+        <v>17.80030340048587</v>
       </c>
       <c r="R9" t="n">
-        <v>16.09357655056119</v>
+        <v>15.95195669566208</v>
       </c>
       <c r="S9" t="n">
-        <v>18.0310359202481</v>
+        <v>18.48431914712054</v>
       </c>
     </row>
     <row r="10">
@@ -1023,55 +1023,55 @@
         <v>199</v>
       </c>
       <c r="C10" t="n">
-        <v>14.55125932466053</v>
+        <v>17.32515557514219</v>
       </c>
       <c r="D10" t="n">
-        <v>10.29382120747885</v>
+        <v>9.545886713611999</v>
       </c>
       <c r="E10" t="n">
-        <v>37.75196774812821</v>
+        <v>26.55789892558693</v>
       </c>
       <c r="F10" t="n">
-        <v>13.02249999999999</v>
+        <v>15.70625000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>8.335000000000001</v>
+        <v>11.53500000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>79.11068195888593</v>
+        <v>90.2108640907513</v>
       </c>
       <c r="I10" t="n">
-        <v>77.17512552629896</v>
+        <v>82.22682044199448</v>
       </c>
       <c r="J10" t="n">
-        <v>63.12289600454023</v>
+        <v>77.42092740338364</v>
       </c>
       <c r="K10" t="n">
-        <v>66.57326790837296</v>
+        <v>71.84705978674424</v>
       </c>
       <c r="L10" t="n">
-        <v>35.01785258978626</v>
+        <v>39.90613987846983</v>
       </c>
       <c r="M10" t="n">
-        <v>25.46566315649368</v>
+        <v>31.56342820417326</v>
       </c>
       <c r="N10" t="n">
-        <v>76.28114118181506</v>
+        <v>84.71754540825648</v>
       </c>
       <c r="O10" t="n">
-        <v>63.29000711012758</v>
+        <v>73.37276402044564</v>
       </c>
       <c r="P10" t="n">
-        <v>20.59078089256755</v>
+        <v>15.72730268272034</v>
       </c>
       <c r="Q10" t="n">
-        <v>17.64003724314817</v>
+        <v>14.23342797453328</v>
       </c>
       <c r="R10" t="n">
-        <v>16.88146494862344</v>
+        <v>12.62790118848821</v>
       </c>
       <c r="S10" t="n">
-        <v>18.69706262348372</v>
+        <v>14.90201899303384</v>
       </c>
     </row>
     <row r="11">
@@ -1084,55 +1084,55 @@
         <v>100</v>
       </c>
       <c r="C11" t="n">
-        <v>17.52247268063871</v>
+        <v>19.37890611723579</v>
       </c>
       <c r="D11" t="n">
-        <v>8.149460637215721</v>
+        <v>10.95492796115531</v>
       </c>
       <c r="E11" t="n">
-        <v>21.25000000000003</v>
+        <v>16.28517085328265</v>
       </c>
       <c r="F11" t="n">
-        <v>14.70000000000001</v>
+        <v>19.05875</v>
       </c>
       <c r="G11" t="n">
-        <v>11.66000000000001</v>
+        <v>16.29625000000001</v>
       </c>
       <c r="H11" t="n">
-        <v>83.25412902673355</v>
+        <v>102.9235152916961</v>
       </c>
       <c r="I11" t="n">
-        <v>71.58910531638176</v>
+        <v>81.00617260431454</v>
       </c>
       <c r="J11" t="n">
-        <v>68.52919086053767</v>
+        <v>87.5128561983895</v>
       </c>
       <c r="K11" t="n">
-        <v>63.73578272838579</v>
+        <v>70.88899773589694</v>
       </c>
       <c r="L11" t="n">
-        <v>43.54595273960601</v>
+        <v>53.44623466625128</v>
       </c>
       <c r="M11" t="n">
-        <v>33.67862823809782</v>
+        <v>42.08622102303794</v>
       </c>
       <c r="N11" t="n">
-        <v>75.6042326857432</v>
+        <v>89.81543575577641</v>
       </c>
       <c r="O11" t="n">
-        <v>63.06048683605288</v>
+        <v>75.87201394453689</v>
       </c>
       <c r="P11" t="n">
-        <v>18.0050365531013</v>
+        <v>15.59633386920283</v>
       </c>
       <c r="Q11" t="n">
-        <v>15.43580159228664</v>
+        <v>15.07946469335257</v>
       </c>
       <c r="R11" t="n">
-        <v>12.44792490375493</v>
+        <v>14.42861071700422</v>
       </c>
       <c r="S11" t="n">
-        <v>17.90206014471826</v>
+        <v>17.18351105540835</v>
       </c>
     </row>
     <row r="12">
@@ -1145,55 +1145,55 @@
         <v>106</v>
       </c>
       <c r="C12" t="n">
-        <v>16.28243799150408</v>
+        <v>26.9391671084671</v>
       </c>
       <c r="D12" t="n">
-        <v>6.371555930591237</v>
+        <v>9.182754136206256</v>
       </c>
       <c r="E12" t="n">
-        <v>22.38104562365379</v>
+        <v>32.91465932553341</v>
       </c>
       <c r="F12" t="n">
-        <v>12.7675</v>
+        <v>14.53</v>
       </c>
       <c r="G12" t="n">
-        <v>10.51875</v>
+        <v>9.747499999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>70.3846574190711</v>
+        <v>79.57700672933106</v>
       </c>
       <c r="I12" t="n">
-        <v>71.81399585039117</v>
+        <v>71.42128534267637</v>
       </c>
       <c r="J12" t="n">
-        <v>60.40281450396165</v>
+        <v>53.98379386445529</v>
       </c>
       <c r="K12" t="n">
-        <v>62.86692294044619</v>
+        <v>63.25345840347388</v>
       </c>
       <c r="L12" t="n">
-        <v>40.07804885470349</v>
+        <v>43.13930922024599</v>
       </c>
       <c r="M12" t="n">
-        <v>33.58943286213687</v>
+        <v>34.73110997362452</v>
       </c>
       <c r="N12" t="n">
-        <v>67.16072140767994</v>
+        <v>71.78527007680614</v>
       </c>
       <c r="O12" t="n">
-        <v>59.65159260237736</v>
+        <v>57.14236606931848</v>
       </c>
       <c r="P12" t="n">
-        <v>19.8746944201318</v>
+        <v>32.76658849513943</v>
       </c>
       <c r="Q12" t="n">
-        <v>16.12941329843631</v>
+        <v>23.35825024642653</v>
       </c>
       <c r="R12" t="n">
-        <v>12.68974289789558</v>
+        <v>12.87555741140571</v>
       </c>
       <c r="S12" t="n">
-        <v>11.21468528832632</v>
+        <v>21.44343426155547</v>
       </c>
     </row>
     <row r="13">
@@ -1206,55 +1206,55 @@
         <v>111</v>
       </c>
       <c r="C13" t="n">
-        <v>10.54601552158919</v>
+        <v>10.31894607479071</v>
       </c>
       <c r="D13" t="n">
-        <v>6.665046641612521</v>
+        <v>6.199462249888377</v>
       </c>
       <c r="E13" t="n">
-        <v>20.18779342723001</v>
+        <v>15.13502198032241</v>
       </c>
       <c r="F13" t="n">
-        <v>14.9025</v>
+        <v>17.91375000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>11.92125</v>
+        <v>15.2025</v>
       </c>
       <c r="H13" t="n">
-        <v>85.80209787645056</v>
+        <v>91.67469661798724</v>
       </c>
       <c r="I13" t="n">
-        <v>81.12336284942828</v>
+        <v>79.41190087134295</v>
       </c>
       <c r="J13" t="n">
-        <v>77.00973964376195</v>
+        <v>85.20856764433962</v>
       </c>
       <c r="K13" t="n">
-        <v>75.11657606680431</v>
+        <v>73.66987172514962</v>
       </c>
       <c r="L13" t="n">
-        <v>38.19031290785663</v>
+        <v>46.59667370102721</v>
       </c>
       <c r="M13" t="n">
-        <v>30.79366818032565</v>
+        <v>39.85285435197836</v>
       </c>
       <c r="N13" t="n">
-        <v>81.65514374489827</v>
+        <v>83.0259748512476</v>
       </c>
       <c r="O13" t="n">
-        <v>74.25967950375222</v>
+        <v>76.81959385469308</v>
       </c>
       <c r="P13" t="n">
-        <v>10.24725321442495</v>
+        <v>7.053341011415911</v>
       </c>
       <c r="Q13" t="n">
-        <v>8.967519590370829</v>
+        <v>7.55340743189477</v>
       </c>
       <c r="R13" t="n">
-        <v>7.613978196004837</v>
+        <v>8.487004502661271</v>
       </c>
       <c r="S13" t="n">
-        <v>9.202457082623473</v>
+        <v>8.222994783064761</v>
       </c>
     </row>
     <row r="14">
@@ -1267,55 +1267,55 @@
         <v>135</v>
       </c>
       <c r="C14" t="n">
-        <v>19.79898773385233</v>
+        <v>19.82538688704793</v>
       </c>
       <c r="D14" t="n">
-        <v>10.95801726674919</v>
+        <v>12.43714885149903</v>
       </c>
       <c r="E14" t="n">
-        <v>34.79035737735677</v>
+        <v>35.9043787714684</v>
       </c>
       <c r="F14" t="n">
-        <v>13.32625000000001</v>
+        <v>17.6525</v>
       </c>
       <c r="G14" t="n">
-        <v>10.67750000000001</v>
+        <v>13.24375000000001</v>
       </c>
       <c r="H14" t="n">
-        <v>78.62887510323418</v>
+        <v>87.09190547921202</v>
       </c>
       <c r="I14" t="n">
-        <v>71.13543420827625</v>
+        <v>77.47257579298625</v>
       </c>
       <c r="J14" t="n">
-        <v>64.62391198310421</v>
+        <v>72.44998274671983</v>
       </c>
       <c r="K14" t="n">
-        <v>62.79530237207238</v>
+        <v>65.61440390645944</v>
       </c>
       <c r="L14" t="n">
-        <v>39.38591118661596</v>
+        <v>52.94572692862003</v>
       </c>
       <c r="M14" t="n">
-        <v>33.77128958153656</v>
+        <v>37.79219496139382</v>
       </c>
       <c r="N14" t="n">
-        <v>73.01926115758774</v>
+        <v>77.81066764910837</v>
       </c>
       <c r="O14" t="n">
-        <v>61.68974793269948</v>
+        <v>66.00615501602861</v>
       </c>
       <c r="P14" t="n">
-        <v>22.29536362901954</v>
+        <v>21.29927853153302</v>
       </c>
       <c r="Q14" t="n">
-        <v>21.25194620489504</v>
+        <v>22.98760497116379</v>
       </c>
       <c r="R14" t="n">
-        <v>20.08279656428454</v>
+        <v>25.46440075000702</v>
       </c>
       <c r="S14" t="n">
-        <v>22.46878628819188</v>
+        <v>21.36379806297339</v>
       </c>
     </row>
     <row r="15">
@@ -1328,55 +1328,55 @@
         <v>990</v>
       </c>
       <c r="C15" t="n">
-        <v>17.69945400239427</v>
+        <v>12.31954396445599</v>
       </c>
       <c r="D15" t="n">
-        <v>9.904300610139034</v>
+        <v>5.990500976257709</v>
       </c>
       <c r="E15" t="n">
-        <v>28.46028239362212</v>
+        <v>29.56875220926124</v>
       </c>
       <c r="F15" t="n">
-        <v>14.17749999999999</v>
+        <v>15.3725</v>
       </c>
       <c r="G15" t="n">
-        <v>10.515</v>
+        <v>11.0275</v>
       </c>
       <c r="H15" t="n">
-        <v>74.46475676452587</v>
+        <v>76.89603370785778</v>
       </c>
       <c r="I15" t="n">
-        <v>65.88247111333939</v>
+        <v>67.74215821775978</v>
       </c>
       <c r="J15" t="n">
-        <v>56.47344508704955</v>
+        <v>63.74362713244361</v>
       </c>
       <c r="K15" t="n">
-        <v>58.52349955359814</v>
+        <v>56.02901034285721</v>
       </c>
       <c r="L15" t="n">
-        <v>43.34166586553867</v>
+        <v>48.10665234663498</v>
       </c>
       <c r="M15" t="n">
-        <v>37.8021163428716</v>
+        <v>39.30012722625717</v>
       </c>
       <c r="N15" t="n">
-        <v>66.88142492501188</v>
+        <v>67.00046641628698</v>
       </c>
       <c r="O15" t="n">
-        <v>55.01420271166347</v>
+        <v>56.2638871746345</v>
       </c>
       <c r="P15" t="n">
-        <v>24.16084126128129</v>
+        <v>24.65199964980351</v>
       </c>
       <c r="Q15" t="n">
-        <v>18.06254645747489</v>
+        <v>20.9644760221328</v>
       </c>
       <c r="R15" t="n">
-        <v>13.56145847973512</v>
+        <v>17.29078048746277</v>
       </c>
       <c r="S15" t="n">
-        <v>17.74367431114702</v>
+        <v>21.02292390639602</v>
       </c>
     </row>
     <row r="16">
@@ -1389,55 +1389,55 @@
         <v>920</v>
       </c>
       <c r="C16" t="n">
-        <v>21.28463985438681</v>
+        <v>25.18271652028316</v>
       </c>
       <c r="D16" t="n">
-        <v>11.88533234201356</v>
+        <v>11.70890274045354</v>
       </c>
       <c r="E16" t="n">
-        <v>33.66436384571112</v>
+        <v>33.5600680204062</v>
       </c>
       <c r="F16" t="n">
-        <v>8.685000000000002</v>
+        <v>12.49625000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>6.79875</v>
+        <v>10</v>
       </c>
       <c r="H16" t="n">
-        <v>69.32892614197915</v>
+        <v>87.14499411899688</v>
       </c>
       <c r="I16" t="n">
-        <v>67.0820393249937</v>
+        <v>76.70886519822857</v>
       </c>
       <c r="J16" t="n">
-        <v>50.11985634456668</v>
+        <v>59.98541489395569</v>
       </c>
       <c r="K16" t="n">
-        <v>50.06246098625197</v>
+        <v>57.68882040742383</v>
       </c>
       <c r="L16" t="n">
-        <v>29.34706118165838</v>
+        <v>36.09016486523717</v>
       </c>
       <c r="M16" t="n">
-        <v>21.50581316760656</v>
+        <v>28.96981187374195</v>
       </c>
       <c r="N16" t="n">
-        <v>67.484257423491</v>
+        <v>80.53609439251447</v>
       </c>
       <c r="O16" t="n">
-        <v>48.40260840078766</v>
+        <v>56.06748166272496</v>
       </c>
       <c r="P16" t="n">
-        <v>27.94559276285958</v>
+        <v>36.06308546917258</v>
       </c>
       <c r="Q16" t="n">
-        <v>26.75111383559634</v>
+        <v>35.7832375323872</v>
       </c>
       <c r="R16" t="n">
-        <v>26.15584837103719</v>
+        <v>35.48641468712599</v>
       </c>
       <c r="S16" t="n">
-        <v>28.27570421788636</v>
+        <v>38.00344805870426</v>
       </c>
     </row>
   </sheetData>

</xml_diff>